<commit_message>
Format chart comparison values in reports
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Dashboard-automation/inputs/Executive-Dashboard-reference.xlsx
+++ b/Dashboard-automation/inputs/Executive-Dashboard-reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AnanthRtr\AnandRtr\Dashboard-automation\Dashboard-automation\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E957B820-F6AF-473F-9B5D-DB5E59050585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CB3759-052E-4B7A-8A7F-E27A69FBA0A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{51C5B8EE-6D16-4030-8EE9-28CD4B5CF6B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{51C5B8EE-6D16-4030-8EE9-28CD4B5CF6B8}"/>
   </bookViews>
   <sheets>
     <sheet name="TG1.1-01-07-2026" sheetId="2" r:id="rId1"/>
@@ -763,10 +763,10 @@
     <t>DL: G14; PV-Syst EP: D14; Ex: J14; RL: L14; PA: H14; GA: I14</t>
   </si>
   <si>
-    <t>DL: S14; PV-Syst EP: P14;  Ex: V14; RL: X14; PA: T14; GA: U14</t>
-  </si>
-  <si>
-    <t>DL: AE14; PV-Syst EP: AB14; Ex: AH14; RL: AJ14; PA: AF14; GA: AG14</t>
+    <t>DL: S14; PV-Syst EP: R14;  Ex: V14; RL: X14; PA: T14; GA: U14</t>
+  </si>
+  <si>
+    <t>DL: AE14; PV-Syst EP: AD14; Ex: AH14; RL: AJ14; PA: AF14; GA: AG14</t>
   </si>
 </sst>
 </file>
@@ -1157,6 +1157,39 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1175,13 +1208,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1213,33 +1240,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1595,12 +1595,12 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="44">
+      <c r="D1" s="24">
         <v>46097</v>
       </c>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -1620,10 +1620,10 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="143" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="23" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="7" t="s">
@@ -1632,7 +1632,7 @@
       <c r="D3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="19" t="s">
         <v>235</v>
       </c>
       <c r="F3" s="8" t="s">
@@ -1643,15 +1643,15 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="105" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="46"/>
-      <c r="B4" s="46"/>
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
       <c r="C4" s="11" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="48" t="s">
+      <c r="E4" s="19" t="s">
         <v>236</v>
       </c>
       <c r="F4" s="8" t="s">
@@ -1662,15 +1662,15 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="149.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="47"/>
-      <c r="B5" s="47"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="11" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="48" t="s">
+      <c r="E5" s="19" t="s">
         <v>237</v>
       </c>
       <c r="F5" s="8" t="s">
@@ -1681,10 +1681,10 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="23" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -1702,15 +1702,15 @@
       <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="46"/>
-      <c r="B7" s="46"/>
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
       <c r="C7" s="7" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="19" t="s">
         <v>185</v>
       </c>
       <c r="F7" s="8" t="s">
@@ -1719,15 +1719,15 @@
       <c r="G7" s="9"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="46"/>
-      <c r="B8" s="46"/>
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
       <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="48" t="s">
+      <c r="E8" s="19" t="s">
         <v>186</v>
       </c>
       <c r="F8" s="8" t="s">
@@ -1736,15 +1736,15 @@
       <c r="G8" s="9"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="46"/>
-      <c r="B9" s="46"/>
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
       <c r="C9" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="48" t="s">
+      <c r="E9" s="19" t="s">
         <v>187</v>
       </c>
       <c r="F9" s="8" t="s">
@@ -1753,15 +1753,15 @@
       <c r="G9" s="9"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="46"/>
-      <c r="B10" s="46"/>
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
       <c r="C10" s="7" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="48" t="s">
+      <c r="E10" s="19" t="s">
         <v>188</v>
       </c>
       <c r="F10" s="8" t="s">
@@ -1770,15 +1770,15 @@
       <c r="G10" s="9"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="46"/>
-      <c r="B11" s="46"/>
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
       <c r="C11" s="7" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="48" t="s">
+      <c r="E11" s="19" t="s">
         <v>189</v>
       </c>
       <c r="F11" s="8" t="s">
@@ -1787,15 +1787,15 @@
       <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="46"/>
-      <c r="B12" s="46"/>
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="7" t="s">
         <v>19</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="48" t="s">
+      <c r="E12" s="19" t="s">
         <v>190</v>
       </c>
       <c r="F12" s="8" t="s">
@@ -1804,15 +1804,15 @@
       <c r="G12" s="9"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="46"/>
-      <c r="B13" s="46"/>
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="48" t="s">
+      <c r="E13" s="19" t="s">
         <v>191</v>
       </c>
       <c r="F13" s="8" t="s">
@@ -1821,15 +1821,15 @@
       <c r="G13" s="9"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="46"/>
-      <c r="B14" s="46"/>
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
       <c r="C14" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="48" t="s">
+      <c r="E14" s="19" t="s">
         <v>192</v>
       </c>
       <c r="F14" s="8" t="s">
@@ -1838,15 +1838,15 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="46"/>
-      <c r="B15" s="46"/>
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" s="19" t="s">
         <v>193</v>
       </c>
       <c r="F15" s="8" t="s">
@@ -1855,15 +1855,15 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="46"/>
-      <c r="B16" s="46"/>
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
       <c r="C16" s="7" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="48" t="s">
+      <c r="E16" s="19" t="s">
         <v>194</v>
       </c>
       <c r="F16" s="8" t="s">
@@ -1872,15 +1872,15 @@
       <c r="G16" s="9"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="46"/>
-      <c r="B17" s="46"/>
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
       <c r="C17" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="48" t="s">
+      <c r="E17" s="19" t="s">
         <v>195</v>
       </c>
       <c r="F17" s="8" t="s">
@@ -1889,15 +1889,15 @@
       <c r="G17" s="9"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="46"/>
-      <c r="B18" s="46"/>
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
       <c r="C18" s="7" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E18" s="48" t="s">
+      <c r="E18" s="19" t="s">
         <v>196</v>
       </c>
       <c r="F18" s="8" t="s">
@@ -1906,15 +1906,15 @@
       <c r="G18" s="9"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="46"/>
-      <c r="B19" s="46"/>
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
       <c r="C19" s="7" t="s">
         <v>26</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="48" t="s">
+      <c r="E19" s="19" t="s">
         <v>197</v>
       </c>
       <c r="F19" s="8" t="s">
@@ -1923,15 +1923,15 @@
       <c r="G19" s="9"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="46"/>
-      <c r="B20" s="46"/>
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="7" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="48" t="s">
+      <c r="E20" s="19" t="s">
         <v>198</v>
       </c>
       <c r="F20" s="8" t="s">
@@ -1940,15 +1940,15 @@
       <c r="G20" s="9"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="46"/>
-      <c r="B21" s="46"/>
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
       <c r="C21" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="48" t="s">
+      <c r="E21" s="19" t="s">
         <v>199</v>
       </c>
       <c r="F21" s="8" t="s">
@@ -1957,15 +1957,15 @@
       <c r="G21" s="9"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="46"/>
-      <c r="B22" s="46"/>
+      <c r="A22" s="21"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="7" t="s">
         <v>29</v>
       </c>
       <c r="D22" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="48" t="s">
+      <c r="E22" s="19" t="s">
         <v>200</v>
       </c>
       <c r="F22" s="8" t="s">
@@ -1974,15 +1974,15 @@
       <c r="G22" s="9"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="46"/>
-      <c r="B23" s="46"/>
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
       <c r="C23" s="7" t="s">
         <v>30</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="48" t="s">
+      <c r="E23" s="19" t="s">
         <v>201</v>
       </c>
       <c r="F23" s="8" t="s">
@@ -1991,15 +1991,15 @@
       <c r="G23" s="9"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
       <c r="C24" s="7" t="s">
         <v>31</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E24" s="48" t="s">
+      <c r="E24" s="19" t="s">
         <v>202</v>
       </c>
       <c r="F24" s="8" t="s">
@@ -2008,15 +2008,15 @@
       <c r="G24" s="9"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="46"/>
-      <c r="B25" s="46"/>
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
       <c r="C25" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="48" t="s">
+      <c r="E25" s="19" t="s">
         <v>203</v>
       </c>
       <c r="F25" s="8" t="s">
@@ -2025,15 +2025,15 @@
       <c r="G25" s="9"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="46"/>
-      <c r="B26" s="46"/>
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
       <c r="C26" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="48" t="s">
+      <c r="E26" s="19" t="s">
         <v>204</v>
       </c>
       <c r="F26" s="8" t="s">
@@ -2042,15 +2042,15 @@
       <c r="G26" s="9"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="46"/>
-      <c r="B27" s="46"/>
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
       <c r="C27" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="48" t="s">
+      <c r="E27" s="19" t="s">
         <v>205</v>
       </c>
       <c r="F27" s="8" t="s">
@@ -2059,15 +2059,15 @@
       <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="46"/>
-      <c r="B28" s="46"/>
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
       <c r="C28" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E28" s="48" t="s">
+      <c r="E28" s="19" t="s">
         <v>206</v>
       </c>
       <c r="F28" s="8" t="s">
@@ -2076,15 +2076,15 @@
       <c r="G28" s="9"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="46"/>
-      <c r="B29" s="46"/>
+      <c r="A29" s="21"/>
+      <c r="B29" s="21"/>
       <c r="C29" s="7" t="s">
         <v>36</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E29" s="48" t="s">
+      <c r="E29" s="19" t="s">
         <v>207</v>
       </c>
       <c r="F29" s="8" t="s">
@@ -2093,15 +2093,15 @@
       <c r="G29" s="9"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="46"/>
-      <c r="B30" s="46"/>
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
       <c r="C30" s="7" t="s">
         <v>37</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="48" t="s">
+      <c r="E30" s="19" t="s">
         <v>208</v>
       </c>
       <c r="F30" s="8" t="s">
@@ -2110,15 +2110,15 @@
       <c r="G30" s="9"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="46"/>
-      <c r="B31" s="46"/>
+      <c r="A31" s="21"/>
+      <c r="B31" s="21"/>
       <c r="C31" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D31" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E31" s="48" t="s">
+      <c r="E31" s="19" t="s">
         <v>209</v>
       </c>
       <c r="F31" s="8" t="s">
@@ -2127,15 +2127,15 @@
       <c r="G31" s="9"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="46"/>
-      <c r="B32" s="46"/>
+      <c r="A32" s="21"/>
+      <c r="B32" s="21"/>
       <c r="C32" s="7" t="s">
         <v>39</v>
       </c>
       <c r="D32" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E32" s="48" t="s">
+      <c r="E32" s="19" t="s">
         <v>210</v>
       </c>
       <c r="F32" s="8" t="s">
@@ -2144,15 +2144,15 @@
       <c r="G32" s="9"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="46"/>
-      <c r="B33" s="46"/>
+      <c r="A33" s="21"/>
+      <c r="B33" s="21"/>
       <c r="C33" s="7" t="s">
         <v>40</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="48" t="s">
+      <c r="E33" s="19" t="s">
         <v>211</v>
       </c>
       <c r="F33" s="8" t="s">
@@ -2161,15 +2161,15 @@
       <c r="G33" s="9"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="46"/>
-      <c r="B34" s="46"/>
+      <c r="A34" s="21"/>
+      <c r="B34" s="21"/>
       <c r="C34" s="7" t="s">
         <v>41</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E34" s="48" t="s">
+      <c r="E34" s="19" t="s">
         <v>212</v>
       </c>
       <c r="F34" s="8" t="s">
@@ -2178,15 +2178,15 @@
       <c r="G34" s="9"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="46"/>
-      <c r="B35" s="46"/>
+      <c r="A35" s="21"/>
+      <c r="B35" s="21"/>
       <c r="C35" s="7" t="s">
         <v>42</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E35" s="48" t="s">
+      <c r="E35" s="19" t="s">
         <v>213</v>
       </c>
       <c r="F35" s="8" t="s">
@@ -2195,15 +2195,15 @@
       <c r="G35" s="9"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="46"/>
-      <c r="B36" s="46"/>
+      <c r="A36" s="21"/>
+      <c r="B36" s="21"/>
       <c r="C36" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E36" s="48" t="s">
+      <c r="E36" s="19" t="s">
         <v>214</v>
       </c>
       <c r="F36" s="8" t="s">
@@ -2212,15 +2212,15 @@
       <c r="G36" s="9"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="46"/>
-      <c r="B37" s="46"/>
+      <c r="A37" s="21"/>
+      <c r="B37" s="21"/>
       <c r="C37" s="7" t="s">
         <v>44</v>
       </c>
       <c r="D37" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="48" t="s">
+      <c r="E37" s="19" t="s">
         <v>215</v>
       </c>
       <c r="F37" s="8" t="s">
@@ -2229,15 +2229,15 @@
       <c r="G37" s="9"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="46"/>
-      <c r="B38" s="46"/>
+      <c r="A38" s="21"/>
+      <c r="B38" s="21"/>
       <c r="C38" s="7" t="s">
         <v>45</v>
       </c>
       <c r="D38" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="48" t="s">
+      <c r="E38" s="19" t="s">
         <v>216</v>
       </c>
       <c r="F38" s="8" t="s">
@@ -2246,15 +2246,15 @@
       <c r="G38" s="9"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="46"/>
-      <c r="B39" s="46"/>
+      <c r="A39" s="21"/>
+      <c r="B39" s="21"/>
       <c r="C39" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D39" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E39" s="48" t="s">
+      <c r="E39" s="19" t="s">
         <v>217</v>
       </c>
       <c r="F39" s="8" t="s">
@@ -2263,15 +2263,15 @@
       <c r="G39" s="9"/>
     </row>
     <row r="40" spans="1:7" ht="17.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="46"/>
-      <c r="B40" s="46"/>
+      <c r="A40" s="21"/>
+      <c r="B40" s="21"/>
       <c r="C40" s="7" t="s">
         <v>47</v>
       </c>
       <c r="D40" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E40" s="48" t="s">
+      <c r="E40" s="19" t="s">
         <v>218</v>
       </c>
       <c r="F40" s="8" t="s">
@@ -2280,15 +2280,15 @@
       <c r="G40" s="9"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A41" s="46"/>
-      <c r="B41" s="46"/>
+      <c r="A41" s="21"/>
+      <c r="B41" s="21"/>
       <c r="C41" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D41" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E41" s="48" t="s">
+      <c r="E41" s="19" t="s">
         <v>219</v>
       </c>
       <c r="F41" s="8" t="s">
@@ -2297,15 +2297,15 @@
       <c r="G41" s="9"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A42" s="46"/>
-      <c r="B42" s="46"/>
+      <c r="A42" s="21"/>
+      <c r="B42" s="21"/>
       <c r="C42" s="7" t="s">
         <v>49</v>
       </c>
       <c r="D42" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E42" s="48" t="s">
+      <c r="E42" s="19" t="s">
         <v>220</v>
       </c>
       <c r="F42" s="8" t="s">
@@ -2314,15 +2314,15 @@
       <c r="G42" s="9"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A43" s="46"/>
-      <c r="B43" s="46"/>
+      <c r="A43" s="21"/>
+      <c r="B43" s="21"/>
       <c r="C43" s="7" t="s">
         <v>50</v>
       </c>
       <c r="D43" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E43" s="48" t="s">
+      <c r="E43" s="19" t="s">
         <v>221</v>
       </c>
       <c r="F43" s="8" t="s">
@@ -2331,15 +2331,15 @@
       <c r="G43" s="9"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A44" s="46"/>
-      <c r="B44" s="46"/>
+      <c r="A44" s="21"/>
+      <c r="B44" s="21"/>
       <c r="C44" s="7" t="s">
         <v>51</v>
       </c>
       <c r="D44" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E44" s="48" t="s">
+      <c r="E44" s="19" t="s">
         <v>222</v>
       </c>
       <c r="F44" s="8" t="s">
@@ -2348,15 +2348,15 @@
       <c r="G44" s="9"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A45" s="46"/>
-      <c r="B45" s="46"/>
+      <c r="A45" s="21"/>
+      <c r="B45" s="21"/>
       <c r="C45" s="7" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E45" s="48" t="s">
+      <c r="E45" s="19" t="s">
         <v>223</v>
       </c>
       <c r="F45" s="8" t="s">
@@ -2365,15 +2365,15 @@
       <c r="G45" s="9"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A46" s="46"/>
-      <c r="B46" s="46"/>
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
       <c r="C46" s="7" t="s">
         <v>53</v>
       </c>
       <c r="D46" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="E46" s="19" t="s">
         <v>224</v>
       </c>
       <c r="F46" s="8" t="s">
@@ -2382,15 +2382,15 @@
       <c r="G46" s="9"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A47" s="46"/>
-      <c r="B47" s="46"/>
+      <c r="A47" s="21"/>
+      <c r="B47" s="21"/>
       <c r="C47" s="7" t="s">
         <v>54</v>
       </c>
       <c r="D47" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E47" s="48" t="s">
+      <c r="E47" s="19" t="s">
         <v>225</v>
       </c>
       <c r="F47" s="8" t="s">
@@ -2399,15 +2399,15 @@
       <c r="G47" s="9"/>
     </row>
     <row r="48" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="46"/>
-      <c r="B48" s="46"/>
+      <c r="A48" s="21"/>
+      <c r="B48" s="21"/>
       <c r="C48" s="7" t="s">
         <v>55</v>
       </c>
       <c r="D48" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E48" s="48" t="s">
+      <c r="E48" s="19" t="s">
         <v>226</v>
       </c>
       <c r="F48" s="8" t="s">
@@ -2416,15 +2416,15 @@
       <c r="G48" s="9"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A49" s="46"/>
-      <c r="B49" s="46"/>
+      <c r="A49" s="21"/>
+      <c r="B49" s="21"/>
       <c r="C49" s="7" t="s">
         <v>56</v>
       </c>
       <c r="D49" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E49" s="48" t="s">
+      <c r="E49" s="19" t="s">
         <v>227</v>
       </c>
       <c r="F49" s="8" t="s">
@@ -2433,15 +2433,15 @@
       <c r="G49" s="9"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A50" s="46"/>
-      <c r="B50" s="46"/>
+      <c r="A50" s="21"/>
+      <c r="B50" s="21"/>
       <c r="C50" s="7" t="s">
         <v>57</v>
       </c>
       <c r="D50" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E50" s="48" t="s">
+      <c r="E50" s="19" t="s">
         <v>228</v>
       </c>
       <c r="F50" s="8" t="s">
@@ -2450,15 +2450,15 @@
       <c r="G50" s="9"/>
     </row>
     <row r="51" spans="1:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="46"/>
-      <c r="B51" s="46"/>
+      <c r="A51" s="21"/>
+      <c r="B51" s="21"/>
       <c r="C51" s="7" t="s">
         <v>58</v>
       </c>
       <c r="D51" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E51" s="48" t="s">
+      <c r="E51" s="19" t="s">
         <v>229</v>
       </c>
       <c r="F51" s="8" t="s">
@@ -2467,15 +2467,15 @@
       <c r="G51" s="9"/>
     </row>
     <row r="52" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="46"/>
-      <c r="B52" s="46"/>
+      <c r="A52" s="21"/>
+      <c r="B52" s="21"/>
       <c r="C52" s="7" t="s">
         <v>59</v>
       </c>
       <c r="D52" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E52" s="48" t="s">
+      <c r="E52" s="19" t="s">
         <v>230</v>
       </c>
       <c r="F52" s="8" t="s">
@@ -2484,15 +2484,15 @@
       <c r="G52" s="9"/>
     </row>
     <row r="53" spans="1:7" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="46"/>
-      <c r="B53" s="46"/>
+      <c r="A53" s="21"/>
+      <c r="B53" s="21"/>
       <c r="C53" s="7" t="s">
         <v>60</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E53" s="48" t="s">
+      <c r="E53" s="19" t="s">
         <v>231</v>
       </c>
       <c r="F53" s="8" t="s">
@@ -2501,15 +2501,15 @@
       <c r="G53" s="9"/>
     </row>
     <row r="54" spans="1:7" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="46"/>
-      <c r="B54" s="46"/>
+      <c r="A54" s="21"/>
+      <c r="B54" s="21"/>
       <c r="C54" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E54" s="48" t="s">
+      <c r="E54" s="19" t="s">
         <v>232</v>
       </c>
       <c r="F54" s="8" t="s">
@@ -2518,15 +2518,15 @@
       <c r="G54" s="9"/>
     </row>
     <row r="55" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="46"/>
-      <c r="B55" s="46"/>
+      <c r="A55" s="21"/>
+      <c r="B55" s="21"/>
       <c r="C55" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E55" s="48" t="s">
+      <c r="E55" s="19" t="s">
         <v>233</v>
       </c>
       <c r="F55" s="8" t="s">
@@ -2535,15 +2535,15 @@
       <c r="G55" s="9"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A56" s="47"/>
-      <c r="B56" s="47"/>
+      <c r="A56" s="22"/>
+      <c r="B56" s="22"/>
       <c r="C56" s="7" t="s">
         <v>63</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E56" s="48" t="s">
+      <c r="E56" s="19" t="s">
         <v>234</v>
       </c>
       <c r="F56" s="8" t="s">
@@ -2552,10 +2552,10 @@
       <c r="G56" s="9"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A57" s="25" t="s">
+      <c r="A57" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B57" s="27" t="s">
+      <c r="B57" s="23" t="s">
         <v>64</v>
       </c>
       <c r="C57" s="7" t="s">
@@ -2573,8 +2573,8 @@
       <c r="G57" s="9"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A58" s="46"/>
-      <c r="B58" s="46"/>
+      <c r="A58" s="21"/>
+      <c r="B58" s="21"/>
       <c r="C58" s="7" t="s">
         <v>66</v>
       </c>
@@ -2590,8 +2590,8 @@
       <c r="G58" s="9"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A59" s="46"/>
-      <c r="B59" s="46"/>
+      <c r="A59" s="21"/>
+      <c r="B59" s="21"/>
       <c r="C59" s="7" t="s">
         <v>67</v>
       </c>
@@ -2607,8 +2607,8 @@
       <c r="G59" s="9"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A60" s="46"/>
-      <c r="B60" s="46"/>
+      <c r="A60" s="21"/>
+      <c r="B60" s="21"/>
       <c r="C60" s="7" t="s">
         <v>68</v>
       </c>
@@ -2624,8 +2624,8 @@
       <c r="G60" s="9"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A61" s="46"/>
-      <c r="B61" s="46"/>
+      <c r="A61" s="21"/>
+      <c r="B61" s="21"/>
       <c r="C61" s="7" t="s">
         <v>69</v>
       </c>
@@ -2641,8 +2641,8 @@
       <c r="G61" s="9"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A62" s="46"/>
-      <c r="B62" s="46"/>
+      <c r="A62" s="21"/>
+      <c r="B62" s="21"/>
       <c r="C62" s="7" t="s">
         <v>70</v>
       </c>
@@ -2658,8 +2658,8 @@
       <c r="G62" s="9"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A63" s="46"/>
-      <c r="B63" s="46"/>
+      <c r="A63" s="21"/>
+      <c r="B63" s="21"/>
       <c r="C63" s="7" t="s">
         <v>71</v>
       </c>
@@ -2675,8 +2675,8 @@
       <c r="G63" s="9"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A64" s="46"/>
-      <c r="B64" s="46"/>
+      <c r="A64" s="21"/>
+      <c r="B64" s="21"/>
       <c r="C64" s="7" t="s">
         <v>72</v>
       </c>
@@ -2692,8 +2692,8 @@
       <c r="G64" s="9"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A65" s="46"/>
-      <c r="B65" s="46"/>
+      <c r="A65" s="21"/>
+      <c r="B65" s="21"/>
       <c r="C65" s="7" t="s">
         <v>73</v>
       </c>
@@ -2709,8 +2709,8 @@
       <c r="G65" s="9"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A66" s="47"/>
-      <c r="B66" s="47"/>
+      <c r="A66" s="22"/>
+      <c r="B66" s="22"/>
       <c r="C66" s="7" t="s">
         <v>74</v>
       </c>
@@ -2726,10 +2726,10 @@
       <c r="G66" s="9"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A67" s="19" t="s">
+      <c r="A67" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B67" s="22" t="s">
+      <c r="B67" s="35" t="s">
         <v>75</v>
       </c>
       <c r="C67" s="7" t="s">
@@ -2747,8 +2747,8 @@
       <c r="G67" s="9"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A68" s="20"/>
-      <c r="B68" s="23"/>
+      <c r="A68" s="33"/>
+      <c r="B68" s="36"/>
       <c r="C68" s="7" t="s">
         <v>77</v>
       </c>
@@ -2764,8 +2764,8 @@
       <c r="G68" s="9"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A69" s="20"/>
-      <c r="B69" s="23"/>
+      <c r="A69" s="33"/>
+      <c r="B69" s="36"/>
       <c r="C69" s="7" t="s">
         <v>78</v>
       </c>
@@ -2781,8 +2781,8 @@
       <c r="G69" s="9"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A70" s="20"/>
-      <c r="B70" s="23"/>
+      <c r="A70" s="33"/>
+      <c r="B70" s="36"/>
       <c r="C70" s="7" t="s">
         <v>79</v>
       </c>
@@ -2798,8 +2798,8 @@
       <c r="G70" s="9"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A71" s="20"/>
-      <c r="B71" s="23"/>
+      <c r="A71" s="33"/>
+      <c r="B71" s="36"/>
       <c r="C71" s="7" t="s">
         <v>80</v>
       </c>
@@ -2815,8 +2815,8 @@
       <c r="G71" s="9"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A72" s="20"/>
-      <c r="B72" s="23"/>
+      <c r="A72" s="33"/>
+      <c r="B72" s="36"/>
       <c r="C72" s="7" t="s">
         <v>81</v>
       </c>
@@ -2832,8 +2832,8 @@
       <c r="G72" s="9"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A73" s="20"/>
-      <c r="B73" s="23"/>
+      <c r="A73" s="33"/>
+      <c r="B73" s="36"/>
       <c r="C73" s="7" t="s">
         <v>82</v>
       </c>
@@ -2849,8 +2849,8 @@
       <c r="G73" s="9"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A74" s="20"/>
-      <c r="B74" s="23"/>
+      <c r="A74" s="33"/>
+      <c r="B74" s="36"/>
       <c r="C74" s="7" t="s">
         <v>83</v>
       </c>
@@ -2866,8 +2866,8 @@
       <c r="G74" s="9"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A75" s="20"/>
-      <c r="B75" s="23"/>
+      <c r="A75" s="33"/>
+      <c r="B75" s="36"/>
       <c r="C75" s="7" t="s">
         <v>84</v>
       </c>
@@ -2883,8 +2883,8 @@
       <c r="G75" s="9"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A76" s="20"/>
-      <c r="B76" s="23"/>
+      <c r="A76" s="33"/>
+      <c r="B76" s="36"/>
       <c r="C76" s="7" t="s">
         <v>85</v>
       </c>
@@ -2900,8 +2900,8 @@
       <c r="G76" s="9"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A77" s="20"/>
-      <c r="B77" s="23"/>
+      <c r="A77" s="33"/>
+      <c r="B77" s="36"/>
       <c r="C77" s="7" t="s">
         <v>86</v>
       </c>
@@ -2917,8 +2917,8 @@
       <c r="G77" s="9"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A78" s="20"/>
-      <c r="B78" s="23"/>
+      <c r="A78" s="33"/>
+      <c r="B78" s="36"/>
       <c r="C78" s="7" t="s">
         <v>87</v>
       </c>
@@ -2934,8 +2934,8 @@
       <c r="G78" s="9"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A79" s="20"/>
-      <c r="B79" s="23"/>
+      <c r="A79" s="33"/>
+      <c r="B79" s="36"/>
       <c r="C79" s="7" t="s">
         <v>88</v>
       </c>
@@ -2951,8 +2951,8 @@
       <c r="G79" s="9"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A80" s="20"/>
-      <c r="B80" s="23"/>
+      <c r="A80" s="33"/>
+      <c r="B80" s="36"/>
       <c r="C80" s="7" t="s">
         <v>89</v>
       </c>
@@ -2968,8 +2968,8 @@
       <c r="G80" s="9"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A81" s="20"/>
-      <c r="B81" s="23"/>
+      <c r="A81" s="33"/>
+      <c r="B81" s="36"/>
       <c r="C81" s="7" t="s">
         <v>90</v>
       </c>
@@ -2985,8 +2985,8 @@
       <c r="G81" s="9"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A82" s="21"/>
-      <c r="B82" s="24"/>
+      <c r="A82" s="34"/>
+      <c r="B82" s="37"/>
       <c r="C82" s="7" t="s">
         <v>65</v>
       </c>
@@ -3005,7 +3005,7 @@
       <c r="A83" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B83" s="22" t="s">
+      <c r="B83" s="35" t="s">
         <v>92</v>
       </c>
       <c r="C83" s="7" t="s">
@@ -3024,7 +3024,7 @@
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="14"/>
-      <c r="B84" s="23"/>
+      <c r="B84" s="36"/>
       <c r="C84" s="7" t="s">
         <v>94</v>
       </c>
@@ -3041,7 +3041,7 @@
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="14"/>
-      <c r="B85" s="23"/>
+      <c r="B85" s="36"/>
       <c r="C85" s="7" t="s">
         <v>84</v>
       </c>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="14"/>
-      <c r="B86" s="23"/>
+      <c r="B86" s="36"/>
       <c r="C86" s="7" t="s">
         <v>87</v>
       </c>
@@ -3075,7 +3075,7 @@
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="14"/>
-      <c r="B87" s="23"/>
+      <c r="B87" s="36"/>
       <c r="C87" s="7" t="s">
         <v>95</v>
       </c>
@@ -3092,7 +3092,7 @@
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="14"/>
-      <c r="B88" s="23"/>
+      <c r="B88" s="36"/>
       <c r="C88" s="7" t="s">
         <v>85</v>
       </c>
@@ -3109,7 +3109,7 @@
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="14"/>
-      <c r="B89" s="23"/>
+      <c r="B89" s="36"/>
       <c r="C89" s="7" t="s">
         <v>82</v>
       </c>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="14"/>
-      <c r="B90" s="23"/>
+      <c r="B90" s="36"/>
       <c r="C90" s="7" t="s">
         <v>96</v>
       </c>
@@ -3143,7 +3143,7 @@
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="14"/>
-      <c r="B91" s="23"/>
+      <c r="B91" s="36"/>
       <c r="C91" s="7" t="s">
         <v>91</v>
       </c>
@@ -3160,7 +3160,7 @@
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="14"/>
-      <c r="B92" s="23"/>
+      <c r="B92" s="36"/>
       <c r="C92" s="7" t="s">
         <v>83</v>
       </c>
@@ -3177,7 +3177,7 @@
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="14"/>
-      <c r="B93" s="23"/>
+      <c r="B93" s="36"/>
       <c r="C93" s="7" t="s">
         <v>80</v>
       </c>
@@ -3193,8 +3193,8 @@
       <c r="G93" s="9"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A94" s="20"/>
-      <c r="B94" s="23"/>
+      <c r="A94" s="33"/>
+      <c r="B94" s="36"/>
       <c r="C94" s="7" t="s">
         <v>86</v>
       </c>
@@ -3210,8 +3210,8 @@
       <c r="G94" s="9"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A95" s="20"/>
-      <c r="B95" s="23"/>
+      <c r="A95" s="33"/>
+      <c r="B95" s="36"/>
       <c r="C95" s="7" t="s">
         <v>90</v>
       </c>
@@ -3227,8 +3227,8 @@
       <c r="G95" s="9"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A96" s="20"/>
-      <c r="B96" s="23"/>
+      <c r="A96" s="33"/>
+      <c r="B96" s="36"/>
       <c r="C96" s="7" t="s">
         <v>97</v>
       </c>
@@ -3244,8 +3244,8 @@
       <c r="G96" s="9"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A97" s="20"/>
-      <c r="B97" s="23"/>
+      <c r="A97" s="33"/>
+      <c r="B97" s="36"/>
       <c r="C97" s="7" t="s">
         <v>98</v>
       </c>
@@ -3261,8 +3261,8 @@
       <c r="G97" s="9"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A98" s="21"/>
-      <c r="B98" s="24"/>
+      <c r="A98" s="34"/>
+      <c r="B98" s="37"/>
       <c r="C98" s="7" t="s">
         <v>65</v>
       </c>
@@ -3278,10 +3278,10 @@
       <c r="G98" s="9"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A99" s="19" t="s">
+      <c r="A99" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B99" s="22" t="s">
+      <c r="B99" s="35" t="s">
         <v>99</v>
       </c>
       <c r="C99" s="7" t="s">
@@ -3299,8 +3299,8 @@
       <c r="G99" s="9"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A100" s="20"/>
-      <c r="B100" s="23"/>
+      <c r="A100" s="33"/>
+      <c r="B100" s="36"/>
       <c r="C100" s="7" t="s">
         <v>102</v>
       </c>
@@ -3316,8 +3316,8 @@
       <c r="G100" s="9"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A101" s="20"/>
-      <c r="B101" s="23"/>
+      <c r="A101" s="33"/>
+      <c r="B101" s="36"/>
       <c r="C101" s="7" t="s">
         <v>104</v>
       </c>
@@ -3333,8 +3333,8 @@
       <c r="G101" s="9"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A102" s="20"/>
-      <c r="B102" s="23"/>
+      <c r="A102" s="33"/>
+      <c r="B102" s="36"/>
       <c r="C102" s="7" t="s">
         <v>106</v>
       </c>
@@ -3350,8 +3350,8 @@
       <c r="G102" s="9"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A103" s="21"/>
-      <c r="B103" s="24"/>
+      <c r="A103" s="34"/>
+      <c r="B103" s="37"/>
       <c r="C103" s="7" t="s">
         <v>108</v>
       </c>
@@ -3367,10 +3367,10 @@
       <c r="G103" s="9"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A104" s="19" t="s">
+      <c r="A104" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B104" s="22" t="s">
+      <c r="B104" s="35" t="s">
         <v>110</v>
       </c>
       <c r="C104" s="7" t="s">
@@ -3388,8 +3388,8 @@
       <c r="G104" s="9"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A105" s="20"/>
-      <c r="B105" s="23"/>
+      <c r="A105" s="33"/>
+      <c r="B105" s="36"/>
       <c r="C105" s="7" t="s">
         <v>113</v>
       </c>
@@ -3405,8 +3405,8 @@
       <c r="G105" s="9"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A106" s="20"/>
-      <c r="B106" s="23"/>
+      <c r="A106" s="33"/>
+      <c r="B106" s="36"/>
       <c r="C106" s="7" t="s">
         <v>115</v>
       </c>
@@ -3422,8 +3422,8 @@
       <c r="G106" s="9"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A107" s="20"/>
-      <c r="B107" s="23"/>
+      <c r="A107" s="33"/>
+      <c r="B107" s="36"/>
       <c r="C107" s="7" t="s">
         <v>117</v>
       </c>
@@ -3439,8 +3439,8 @@
       <c r="G107" s="9"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A108" s="21"/>
-      <c r="B108" s="24"/>
+      <c r="A108" s="34"/>
+      <c r="B108" s="37"/>
       <c r="C108" s="7" t="s">
         <v>119</v>
       </c>
@@ -3456,49 +3456,49 @@
       <c r="G108" s="9"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A109" s="25" t="s">
+      <c r="A109" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B109" s="27" t="s">
+      <c r="B109" s="23" t="s">
         <v>121</v>
       </c>
       <c r="C109" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="D109" s="29" t="s">
+      <c r="D109" s="40" t="s">
         <v>123</v>
       </c>
-      <c r="E109" s="30"/>
-      <c r="F109" s="30"/>
-      <c r="G109" s="31"/>
+      <c r="E109" s="41"/>
+      <c r="F109" s="41"/>
+      <c r="G109" s="42"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A110" s="26"/>
-      <c r="B110" s="28"/>
+      <c r="A110" s="38"/>
+      <c r="B110" s="39"/>
       <c r="C110" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="D110" s="32"/>
-      <c r="E110" s="33"/>
-      <c r="F110" s="33"/>
-      <c r="G110" s="34"/>
+      <c r="D110" s="43"/>
+      <c r="E110" s="44"/>
+      <c r="F110" s="44"/>
+      <c r="G110" s="45"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A111" s="26"/>
-      <c r="B111" s="28"/>
+      <c r="A111" s="38"/>
+      <c r="B111" s="39"/>
       <c r="C111" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="D111" s="35"/>
-      <c r="E111" s="36"/>
-      <c r="F111" s="36"/>
-      <c r="G111" s="37"/>
+      <c r="D111" s="46"/>
+      <c r="E111" s="47"/>
+      <c r="F111" s="47"/>
+      <c r="G111" s="48"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A112" s="38" t="s">
+      <c r="A112" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B112" s="41" t="s">
+      <c r="B112" s="29" t="s">
         <v>126</v>
       </c>
       <c r="C112" s="16" t="s">
@@ -3516,8 +3516,8 @@
       <c r="G112" s="9"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A113" s="39"/>
-      <c r="B113" s="42"/>
+      <c r="A113" s="27"/>
+      <c r="B113" s="30"/>
       <c r="C113" s="16" t="s">
         <v>129</v>
       </c>
@@ -3533,8 +3533,8 @@
       <c r="G113" s="9"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A114" s="39"/>
-      <c r="B114" s="42"/>
+      <c r="A114" s="27"/>
+      <c r="B114" s="30"/>
       <c r="C114" s="16" t="s">
         <v>131</v>
       </c>
@@ -3550,8 +3550,8 @@
       <c r="G114" s="9"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A115" s="39"/>
-      <c r="B115" s="42"/>
+      <c r="A115" s="27"/>
+      <c r="B115" s="30"/>
       <c r="C115" s="16" t="s">
         <v>69</v>
       </c>
@@ -3567,8 +3567,8 @@
       <c r="G115" s="9"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A116" s="39"/>
-      <c r="B116" s="42"/>
+      <c r="A116" s="27"/>
+      <c r="B116" s="30"/>
       <c r="C116" s="16" t="s">
         <v>73</v>
       </c>
@@ -3584,8 +3584,8 @@
       <c r="G116" s="9"/>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A117" s="39"/>
-      <c r="B117" s="42"/>
+      <c r="A117" s="27"/>
+      <c r="B117" s="30"/>
       <c r="C117" s="16" t="s">
         <v>97</v>
       </c>
@@ -3601,8 +3601,8 @@
       <c r="G117" s="9"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A118" s="39"/>
-      <c r="B118" s="42"/>
+      <c r="A118" s="27"/>
+      <c r="B118" s="30"/>
       <c r="C118" s="16" t="s">
         <v>98</v>
       </c>
@@ -3618,8 +3618,8 @@
       <c r="G118" s="9"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A119" s="40"/>
-      <c r="B119" s="43"/>
+      <c r="A119" s="28"/>
+      <c r="B119" s="31"/>
       <c r="C119" s="16" t="s">
         <v>137</v>
       </c>
@@ -3636,13 +3636,7 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A57:A66"/>
-    <mergeCell ref="B57:B66"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="A6:A56"/>
-    <mergeCell ref="B6:B56"/>
+    <mergeCell ref="D109:G111"/>
     <mergeCell ref="A112:A119"/>
     <mergeCell ref="B112:B119"/>
     <mergeCell ref="A67:A82"/>
@@ -3655,8 +3649,15 @@
     <mergeCell ref="B104:B108"/>
     <mergeCell ref="A109:A111"/>
     <mergeCell ref="B109:B111"/>
-    <mergeCell ref="D109:G111"/>
+    <mergeCell ref="A57:A66"/>
+    <mergeCell ref="B57:B66"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="A6:A56"/>
+    <mergeCell ref="B6:B56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>